<commit_message>
add formatation do d column
</commit_message>
<xml_diff>
--- a/analise_formatada.xlsx
+++ b/analise_formatada.xlsx
@@ -460,12 +460,12 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Afirmação</t>
+          <t>Prática</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>Atributo</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -504,12 +504,12 @@
       <c r="C2" s="2" t="n"/>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>Direta Média</t>
+          <t>Média</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>Indireta Média</t>
+          <t>Média</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
@@ -524,12 +524,12 @@
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
-          <t>Direta Média</t>
+          <t>Média</t>
         </is>
       </c>
       <c r="I2" s="1" t="inlineStr">
         <is>
-          <t>Indireta Média</t>
+          <t>Média</t>
         </is>
       </c>
       <c r="J2" s="1" t="inlineStr">
@@ -544,12 +544,12 @@
       </c>
       <c r="L2" s="1" t="inlineStr">
         <is>
-          <t>Direta Média</t>
+          <t>Média</t>
         </is>
       </c>
       <c r="M2" s="1" t="inlineStr">
         <is>
-          <t>Indireta Média</t>
+          <t>Média</t>
         </is>
       </c>
       <c r="N2" s="1" t="inlineStr">
@@ -596,7 +596,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>(0.5668202764976958, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>(0.046153846153846156, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -636,7 +636,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>(-0.021592442645074223, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>(0.511520737327189, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>(-0.028846153846153848, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>(0.07422402159244265, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -740,7 +740,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>(0.6589861751152074, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -760,7 +760,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>(0.0125, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -780,7 +780,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>(0.0951417004048583, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -812,7 +812,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>(0.4093701996927803, 'medium')</t>
+          <t>(+)</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -832,7 +832,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>(0.04326923076923077, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>(0.0931174089068826, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -889,7 +889,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>(0.49615975422427033, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -909,7 +909,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>(-0.0057692307692307696, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>(0.058029689608636977, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>(0.5092165898617511, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -981,7 +981,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>(-0.09615384615384616, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -1001,7 +1001,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>(-0.0708502024291498, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>(0.5837173579109063, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>(-0.1778846153846154, 'small')</t>
+          <t>(-)</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>(0.004723346828609987, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -1105,7 +1105,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>(0.49539170506912444, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>(-0.04038461538461539, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>(0.11336032388663968, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -1182,7 +1182,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>(0.46927803379416283, 'medium')</t>
+          <t>(+)</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>(-0.025961538461538463, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>(-0.012145748987854251, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>(0.46006144393241166, 'medium')</t>
+          <t>(+)</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>(-0.009615384615384616, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -1294,7 +1294,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>(-0.150472334682861, 'small')</t>
+          <t>(-)</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>(0.4539170506912442, 'medium')</t>
+          <t>(+)</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1346,7 +1346,7 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>(-0.13942307692307693, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>(-0.001349527665317139, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -1398,7 +1398,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>(0.5353302611367128, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>(-0.025, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -1438,7 +1438,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>(0.07354925775978408, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -1475,7 +1475,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>(0.4646697388632873, 'medium')</t>
+          <t>(+)</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1495,7 +1495,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>(0.05480769230769231, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -1515,7 +1515,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>(0.1329284750337382, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -1547,7 +1547,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>(0.423963133640553, 'medium')</t>
+          <t>(+)</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>(-0.041346153846153845, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -1587,7 +1587,7 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>(-0.19973009446693657, 'small')</t>
+          <t>(-)</t>
         </is>
       </c>
     </row>
@@ -1619,7 +1619,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>(0.48540706605222733, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>(-0.13365384615384615, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -1659,7 +1659,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>(0.010121457489878543, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -1691,7 +1691,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>(0.4554531490015361, 'medium')</t>
+          <t>(+)</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1711,7 +1711,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>(0.03365384615384615, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>(0.09244264507422402, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -1768,7 +1768,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>(0.5384024577572964, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1788,7 +1788,7 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>(-0.058653846153846154, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>(0.07489878542510121, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>(0.5046082949308756, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>(0.0009615384615384616, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>(-0.07017543859649122, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>(0.6290322580645161, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1932,7 +1932,7 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>(-0.07403846153846154, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -1952,7 +1952,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>(0.02631578947368421, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -1984,7 +1984,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>(0.4485407066052227, 'medium')</t>
+          <t>(+)</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -2004,7 +2004,7 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>(0.014423076923076924, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
@@ -2024,7 +2024,7 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>(0.09851551956815115, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2061,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>(0.6290322580645161, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -2081,7 +2081,7 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>(-0.18557692307692308, 'small')</t>
+          <t>(-)</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>(0.016869095816464237, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -2133,7 +2133,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>(0.5522273425499232, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -2153,7 +2153,7 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>(-0.23365384615384616, 'small')</t>
+          <t>(-)</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
@@ -2173,7 +2173,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>(-0.04116059379217274, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>(0.5468509984639017, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -2225,7 +2225,7 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>(-0.06923076923076923, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
@@ -2245,7 +2245,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>(0.11740890688259109, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -2277,7 +2277,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>(0.4324116743471582, 'medium')</t>
+          <t>(+)</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>(0.08846153846153847, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
@@ -2317,7 +2317,7 @@
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>(0.26653171390013497, 'small')</t>
+          <t>(-)</t>
         </is>
       </c>
     </row>
@@ -2354,7 +2354,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>(0.49923195084485406, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>(-0.12980769230769232, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>(0.09109311740890688, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>(0.5691244239631337, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -2446,7 +2446,7 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>(-0.0028846153846153848, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>(-0.04723346828609987, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -2498,7 +2498,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>(0.5606758832565284, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2518,7 +2518,7 @@
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>(-0.2644230769230769, 'small')</t>
+          <t>(-)</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
@@ -2538,7 +2538,7 @@
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>(-0.0310391363022942, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -2570,7 +2570,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>(0.41397849462365593, 'medium')</t>
+          <t>(+)</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -2590,7 +2590,7 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>(0.016346153846153847, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
@@ -2610,7 +2610,7 @@
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>(0.10323886639676114, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -2647,7 +2647,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>(0.5345622119815668, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>(-0.07307692307692308, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
@@ -2687,7 +2687,7 @@
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>(0.05398110661268556, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -2719,7 +2719,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>(0.5768049155145929, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -2739,7 +2739,7 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>(-0.015384615384615385, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
@@ -2759,7 +2759,7 @@
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>(-0.0020242914979757085, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -2791,7 +2791,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>(0.6190476190476191, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -2811,7 +2811,7 @@
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>(-0.15096153846153845, 'small')</t>
+          <t>(-)</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>(0.020917678812415654, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -2863,7 +2863,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>(0.500768049155146, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>(0.026923076923076925, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>(0.044534412955465584, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -2940,7 +2940,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>(0.5714285714285714, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -2960,7 +2960,7 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>(-0.07211538461538461, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
@@ -2980,7 +2980,7 @@
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>(-0.1592442645074224, 'small')</t>
+          <t>(-)</t>
         </is>
       </c>
     </row>
@@ -3012,7 +3012,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>(0.5445468509984639, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -3032,7 +3032,7 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>(0.08942307692307692, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
@@ -3052,7 +3052,7 @@
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>(-0.08434547908232119, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -3084,7 +3084,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>(0.5675883256528418, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -3104,7 +3104,7 @@
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>(-0.0057692307692307696, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
@@ -3124,7 +3124,7 @@
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>(-0.014844804318488529, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -3156,7 +3156,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>(0.47081413210445466, 'medium')</t>
+          <t>(+)</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -3176,7 +3176,7 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>(0.10192307692307692, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
@@ -3196,7 +3196,7 @@
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>(0.13022941970310392, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>(0.5460829493087558, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -3253,7 +3253,7 @@
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>(-0.0028846153846153848, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
@@ -3273,7 +3273,7 @@
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>(-0.12010796221322537, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -3305,7 +3305,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>(0.5952380952380952, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -3325,7 +3325,7 @@
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>(0.04423076923076923, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
@@ -3345,7 +3345,7 @@
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>(-0.11740890688259109, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>(0.6996927803379416, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -3397,7 +3397,7 @@
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>(-0.17211538461538461, 'small')</t>
+          <t>(-)</t>
         </is>
       </c>
       <c r="L41" s="2" t="inlineStr">
@@ -3417,7 +3417,7 @@
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>(0.0310391363022942, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -3449,7 +3449,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>(0.5476190476190477, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -3469,7 +3469,7 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>(-0.0673076923076923, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
@@ -3489,7 +3489,7 @@
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>(0.05263157894736842, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>(0.2887864823348694, 'small')</t>
+          <t>(-)</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -3546,7 +3546,7 @@
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>(-0.08269230769230769, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
@@ -3566,7 +3566,7 @@
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>(0.10796221322537113, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -3598,7 +3598,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>(0.47081413210445466, 'medium')</t>
+          <t>(+)</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -3618,7 +3618,7 @@
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>(0.0, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr">
@@ -3638,7 +3638,7 @@
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>(-0.0728744939271255, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -3670,7 +3670,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>(0.4062980030721966, 'medium')</t>
+          <t>(+)</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -3690,7 +3690,7 @@
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>(-0.19903846153846153, 'small')</t>
+          <t>(-)</t>
         </is>
       </c>
       <c r="L45" s="2" t="inlineStr">
@@ -3710,7 +3710,7 @@
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>(0.038461538461538464, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -3742,7 +3742,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>(0.4508448540706605, 'medium')</t>
+          <t>(+)</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -3762,7 +3762,7 @@
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>(0.052884615384615384, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr">
@@ -3782,7 +3782,7 @@
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>(0.09919028340080972, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -3819,7 +3819,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>(0.3778801843317972, 'medium')</t>
+          <t>(+)</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>(-0.10961538461538461, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L47" s="2" t="inlineStr">
@@ -3859,7 +3859,7 @@
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>(-0.2483130904183536, 'small')</t>
+          <t>(-)</t>
         </is>
       </c>
     </row>
@@ -3891,7 +3891,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>(0.46390168970814133, 'medium')</t>
+          <t>(+)</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -3911,7 +3911,7 @@
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>(-0.046153846153846156, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr">
@@ -3931,7 +3931,7 @@
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>(-0.31309041835357626, 'small')</t>
+          <t>(-)</t>
         </is>
       </c>
     </row>
@@ -3963,7 +3963,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>(0.3717357910906298, 'medium')</t>
+          <t>(+)</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>(-0.28173076923076923, 'small')</t>
+          <t>(-)</t>
         </is>
       </c>
       <c r="L49" s="2" t="inlineStr">
@@ -4003,7 +4003,7 @@
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>(-0.09446693657219973, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -4035,7 +4035,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>(0.4500768049155146, 'medium')</t>
+          <t>(+)</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -4055,7 +4055,7 @@
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>(0.11923076923076924, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L50" s="2" t="inlineStr">
@@ -4075,7 +4075,7 @@
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>(0.13765182186234817, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -4112,7 +4112,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>(0.5821812596006144, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -4132,7 +4132,7 @@
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>(-0.03653846153846154, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L51" s="2" t="inlineStr">
@@ -4152,7 +4152,7 @@
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>(-0.13225371120107962, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -4184,7 +4184,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>(0.6566820276497696, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -4204,7 +4204,7 @@
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>(-0.08365384615384615, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr">
@@ -4224,7 +4224,7 @@
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>(-0.08502024291497975, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -4256,7 +4256,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>(0.6451612903225806, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -4276,7 +4276,7 @@
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>(-0.14134615384615384, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L53" s="2" t="inlineStr">
@@ -4296,7 +4296,7 @@
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>(0.1329284750337382, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>(0.6505376344086021, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -4348,7 +4348,7 @@
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>(-0.08173076923076923, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L54" s="2" t="inlineStr">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>(0.038461538461538464, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -4405,7 +4405,7 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>(0.4162826420890937, 'medium')</t>
+          <t>(+)</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -4425,7 +4425,7 @@
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>(0.11634615384615385, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L55" s="2" t="inlineStr">
@@ -4445,7 +4445,7 @@
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>(-0.018893387314439947, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -4477,7 +4477,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>(0.49001536098310294, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -4497,7 +4497,7 @@
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>(0.0125, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L56" s="2" t="inlineStr">
@@ -4517,7 +4517,7 @@
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>(-0.09851551956815115, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -4549,7 +4549,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>(0.4915514592933948, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4569,7 +4569,7 @@
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>(-0.11538461538461539, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L57" s="2" t="inlineStr">
@@ -4589,7 +4589,7 @@
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>(-0.02631578947368421, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>(0.5906298003072197, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -4641,7 +4641,7 @@
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>(-0.025961538461538463, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L58" s="2" t="inlineStr">
@@ -4661,7 +4661,7 @@
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>(0.17071524966261808, 'small')</t>
+          <t>(-)</t>
         </is>
       </c>
     </row>
@@ -4698,7 +4698,7 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>(0.5368663594470046, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -4718,7 +4718,7 @@
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>(-0.03173076923076923, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L59" s="2" t="inlineStr">
@@ -4738,7 +4738,7 @@
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>(0.09716599190283401, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -4770,7 +4770,7 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>(0.6397849462365591, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -4790,7 +4790,7 @@
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>(0.0057692307692307696, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L60" s="2" t="inlineStr">
@@ -4810,7 +4810,7 @@
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>(0.011470985155195682, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -4842,7 +4842,7 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>(0.619815668202765, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -4862,7 +4862,7 @@
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>(-0.1, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L61" s="2" t="inlineStr">
@@ -4882,7 +4882,7 @@
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>(0.13832658569500675, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -4914,7 +4914,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>(0.5422427035330261, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -4934,7 +4934,7 @@
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>(0.06538461538461539, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L62" s="2" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>(0.10526315789473684, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>(0.522273425499232, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -5011,7 +5011,7 @@
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>(0.07115384615384615, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L63" s="2" t="inlineStr">
@@ -5031,7 +5031,7 @@
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>(0.20512820512820512, 'small')</t>
+          <t>(-)</t>
         </is>
       </c>
     </row>
@@ -5063,7 +5063,7 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>(0.6221198156682027, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -5083,7 +5083,7 @@
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>(-0.15096153846153845, 'small')</t>
+          <t>(-)</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr">
@@ -5103,7 +5103,7 @@
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>(0.1417004048582996, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -5135,7 +5135,7 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>(0.6758832565284179, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -5155,7 +5155,7 @@
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>(-0.19134615384615383, 'small')</t>
+          <t>(-)</t>
         </is>
       </c>
       <c r="L65" s="2" t="inlineStr">
@@ -5175,7 +5175,7 @@
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>(0.13900134952766532, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>
@@ -5207,7 +5207,7 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>(0.5138248847926268, 'large')</t>
+          <t>(+)*</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
@@ -5227,7 +5227,7 @@
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>(-0.007692307692307693, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
       <c r="L66" s="2" t="inlineStr">
@@ -5247,7 +5247,7 @@
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>(0.09244264507422402, 'negligible')</t>
+          <t>(-)*</t>
         </is>
       </c>
     </row>

</xml_diff>